<commit_message>
E:\anaconda3\Scripts\activate && conda activate py312
</commit_message>
<xml_diff>
--- a/output/P11.xlsx
+++ b/output/P11.xlsx
@@ -3933,15 +3933,16 @@
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
-          <t>User</t>
+          <t>Assistant</t>
         </is>
       </c>
       <c r="C7" s="1" t="inlineStr">
         <is>
-          <t>Prompt</t>
-        </is>
-      </c>
-      <c r="D7" s="1" t="inlineStr">
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D7" s="1" t="inlineStr"/>
+      <c r="E7" s="1" t="inlineStr">
         <is>
           <t>Base directory for this skill: /tmp/claude-1000/bundled-skills/2.1.245/4a8706fc0ed187700741d073ddc62565/dataviz
 # Data Visualization
@@ -4041,7 +4042,6 @@
 | `scripts/validate_palette.js` | Runnable six-checks validator (run it; don't eyeball) |</t>
         </is>
       </c>
-      <c r="E7" s="1" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">

</xml_diff>